<commit_message>
Add Phase 2B Dual-Backbone RGB-Thermal Fusion (v35) with Gated Attention
</commit_message>
<xml_diff>
--- a/results/results_highlighted.xlsx
+++ b/results/results_highlighted.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P106"/>
+  <dimension ref="A1:P108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7065,6 +7065,130 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>v34</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>v34_early_fusion (Early Fusion 4ch + 100ep Cosine LR)</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>models/v34_early_fusion</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="F107" s="2" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="G107" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H107" s="2" t="n">
+        <v>0.842</v>
+      </c>
+      <c r="I107" s="2" t="n">
+        <v>0.5974</v>
+      </c>
+      <c r="J107" s="2" t="n">
+        <v>0.8263</v>
+      </c>
+      <c r="K107" s="2" t="n">
+        <v>0.7761</v>
+      </c>
+      <c r="L107" s="2" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="M107" s="2" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="N107" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:05:49</t>
+        </is>
+      </c>
+      <c r="O107" s="2" t="inlineStr">
+        <is>
+          <t>Early fusion 4-channel [R,G,B,T_gray]. Weight surgery: 4th ch = mean(RGB) from yolov8n.pt</t>
+        </is>
+      </c>
+      <c r="P107" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>v34_eval</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>v34_early_fusion (Early Fusion) [Official Test]</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>models/v34_early_fusion</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="F108" s="2" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="G108" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H108" s="2" t="n">
+        <v>0.8368</v>
+      </c>
+      <c r="I108" s="2" t="n">
+        <v>0.5867</v>
+      </c>
+      <c r="J108" s="2" t="n">
+        <v>0.8176</v>
+      </c>
+      <c r="K108" s="2" t="n">
+        <v>0.8247</v>
+      </c>
+      <c r="L108" s="2" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="M108" s="2" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="N108" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:05:50</t>
+        </is>
+      </c>
+      <c r="O108" s="2" t="inlineStr">
+        <is>
+          <t>Official test split evaluation on 4-channel fusion dataset (108 images)</t>
+        </is>
+      </c>
+      <c r="P108" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Log Phase 2B Dual-Backbone Gated Fusion final 100-epoch results
</commit_message>
<xml_diff>
--- a/results/results_highlighted.xlsx
+++ b/results/results_highlighted.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P108"/>
+  <dimension ref="A1:P110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7189,6 +7189,130 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>v35</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>v35_dual_fusion (Dual-Backbone Gated Fusion + 100ep Cosine LR)</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>models/v35_dual_fusion</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="F109" s="2" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="G109" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H109" s="2" t="n">
+        <v>0.8773</v>
+      </c>
+      <c r="I109" s="2" t="n">
+        <v>0.6351</v>
+      </c>
+      <c r="J109" s="2" t="n">
+        <v>0.8681</v>
+      </c>
+      <c r="K109" s="2" t="n">
+        <v>0.8300999999999999</v>
+      </c>
+      <c r="L109" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M109" s="2" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="N109" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:59:19</t>
+        </is>
+      </c>
+      <c r="O109" s="2" t="inlineStr">
+        <is>
+          <t>Dual-stream RGB + Thermal backbones with multi-scale GatedFusion at P3, P4, P5. 6-channel input.</t>
+        </is>
+      </c>
+      <c r="P109" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>v35_eval</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>v35_dual_fusion (Dual-Backbone Gated Fusion) [Official Test]</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>models/v35_dual_fusion</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="F110" s="2" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="G110" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H110" s="2" t="n">
+        <v>0.8754</v>
+      </c>
+      <c r="I110" s="2" t="n">
+        <v>0.6484</v>
+      </c>
+      <c r="J110" s="2" t="n">
+        <v>0.9068000000000001</v>
+      </c>
+      <c r="K110" s="2" t="n">
+        <v>0.8105</v>
+      </c>
+      <c r="L110" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M110" s="2" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="N110" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:59:19</t>
+        </is>
+      </c>
+      <c r="O110" s="2" t="inlineStr">
+        <is>
+          <t>Official test split evaluation on 6-channel dual fusion dataset (108 images)</t>
+        </is>
+      </c>
+      <c r="P110" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>